<commit_message>
Add The Ride Up playlist — amped Eminem-heavy sing-along rap for the drive up
67 tracks / 4h 41m of windows-down sing-along rap (10th playlist).
Ten Eminem cuts plus five features, validated zero-duplicate against
all 553 existing tracks. Adds per-playlist max_artist override to the
generator so an intentionally artist-heavy list can pass validation;
regenerates all output deliverables including the Soundiiz import CSV.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CpaEpUJu8thEfgbW4uKELZ
</commit_message>
<xml_diff>
--- a/crystal-springs-trip/output/master_playlist.xlsx
+++ b/crystal-springs-trip/output/master_playlist.xlsx
@@ -18,6 +18,7 @@
     <sheet name="Airbnb Morning" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Airbnb Evening" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="Trip Anthem" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="The Ride Up" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -439,10 +440,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="4" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
     <col width="42" customWidth="1" min="3" max="3"/>
     <col width="7" customWidth="1" min="4" max="4"/>
@@ -734,24 +735,52 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
-    <row r="12">
-      <c r="A12" t="inlineStr"/>
-      <c r="B12" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Pedal Down</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>67</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>4h 41m</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>4h 40m</t>
+        </is>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="n">
-        <v>553</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>36h 01m</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr"/>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="n">
+        <v>620</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>40h 42m</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3504,13 +3533,1736 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E68"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="29" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Track #</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Artist</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Song</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Length</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Genre</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Meek Mill</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Dreams and Nightmares</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>3:56</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Eminem feat. Juice WRLD</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Godzilla</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>3:31</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Jay-Z &amp; Kanye West</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Ni**as in Paris</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>3:39</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Eminem</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>4:11</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Wiz Khalifa</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Black and Yellow</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>3:37</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Kanye West</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Stronger</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>5:12</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>50 Cent feat. Eminem &amp; Tony Yayo</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Patiently Waiting</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>4:48</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>M.O.P.</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Ante Up</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>3:56</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Lil Wayne feat. Cory Gunz</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>6 Foot 7 Foot</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>4:09</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Bad Meets Evil</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Fast Lane</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>4:10</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Macklemore &amp; Ryan Lewis feat. Ray Dalton</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Can't Hold Us</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>4:18</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Eminem feat. Rihanna</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>The Monster</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>4:10</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Flo Rida feat. T-Pain</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>3:50</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>J-Kwon</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Tipsy</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>4:04</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>D12</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Purple Pills</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>5:00</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>The Game feat. 50 Cent</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Hate It or Love It</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>3:26</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Nelly feat. P. Diddy &amp; Murphy Lee</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Shake Ya Tailfeather</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>4:53</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Eminem</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Just Lose It</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>4:08</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Ludacris</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Get Back</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>4:30</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Clipse</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Grindin'</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>4:30</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>P. Diddy feat. Black Rob &amp; Mark Curry</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Bad Boy for Life</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>3:42</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Eminem feat. Dr. Dre</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Guilty Conscience</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>3:19</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Cam'ron feat. Juelz Santana</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Oh Boy</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>3:34</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>50 Cent feat. Justin Timberlake &amp; Timbaland</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Ayo Technology</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>4:07</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Akon feat. Eminem</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Smack That</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>3:33</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Jim Jones</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>We Fly High</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>4:01</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>G-Unit</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Stunt 101</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>4:04</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Sir Mix-a-Lot</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Baby Got Back</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>4:22</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Vanilla Ice</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Ice Ice Baby</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>4:31</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>MC Hammer</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>U Can't Touch This</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>4:17</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Kris Kross</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Jump</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>3:16</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Naughty by Nature</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Hip Hop Hooray</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>4:26</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Run-DMC</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>It's Tricky</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>3:03</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Beastie Boys</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Brass Monkey</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>2:37</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Rob Base &amp; DJ E-Z Rock</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>It Takes Two</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>4:57</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Luniz feat. Michael Marshall</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>I Got 5 on It</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>4:14</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Eminem feat. Dido</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Stan</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>6:44</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Xzibit</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>3:47</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Fat Joe &amp; Remy Ma feat. French Montana &amp; Infared</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>All the Way Up</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>3:36</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Rick Ross feat. Styles P</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>B.M.F. (Blowin' Money Fast)</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>4:15</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Eminem</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Like Toy Soldiers</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>4:56</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Asher Roth</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>I Love College</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>4:01</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Soulja Boy</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Crank That (Soulja Boy)</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>3:42</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Macklemore &amp; Ryan Lewis feat. Wanz</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Thrift Shop</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>3:55</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Jay-Z feat. Eminem</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Renegade</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>5:38</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Travis Scott</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>SICKO MODE</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>5:12</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Post Malone feat. Quavo</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>3:40</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Drake feat. Lil Wayne</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>The Motto</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>3:01</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Kanye West feat. Rihanna &amp; Kid Cudi</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>All of the Lights</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>4:59</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Big Sean feat. E-40</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>I Don't Fuck with You</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>4:44</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Kanye West</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Heartless</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>3:31</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Eminem feat. Lil Wayne</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>No Love</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>5:00</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Kid Cudi</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Day 'N' Nite</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>3:42</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Drake</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Started From the Bottom</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>2:53</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>DJ Khaled feat. Drake, Rick Ross &amp; Lil Wayne</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>I'm On One</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>4:56</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>B.o.B feat. Hayley Williams &amp; Eminem</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Airplanes, Pt. II</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>4:20</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Jay-Z feat. Rihanna &amp; Kanye West</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Run This Town</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>4:27</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Nelly</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>E.I.</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>4:47</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Juvenile feat. Soulja Slim</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Slow Motion</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>4:10</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Outkast</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Roses</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>6:09</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Linkin Park &amp; Jay-Z</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Numb / Encore</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>3:25</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Papa Roach</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Last Resort</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>3:20</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Rock</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Too $hort</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Blow the Whistle</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>2:46</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Bad Meets Evil feat. Bruno Mars</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Lighters</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>5:04</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Drake feat. Kanye West, Lil Wayne &amp; Eminem</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Forever</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>5:57</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Eminem feat. Rihanna</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Love the Way You Lie</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>4:23</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Eminem</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Not Afraid</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>4:08</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F554"/>
+  <dimension ref="A1:F621"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -20140,6 +21892,2016 @@
       <c r="F554" t="inlineStr">
         <is>
           <t>Rock</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B555" t="n">
+        <v>1</v>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>Meek Mill</t>
+        </is>
+      </c>
+      <c r="D555" t="inlineStr">
+        <is>
+          <t>Dreams and Nightmares</t>
+        </is>
+      </c>
+      <c r="E555" t="inlineStr">
+        <is>
+          <t>3:56</t>
+        </is>
+      </c>
+      <c r="F555" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B556" t="n">
+        <v>2</v>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>Eminem feat. Juice WRLD</t>
+        </is>
+      </c>
+      <c r="D556" t="inlineStr">
+        <is>
+          <t>Godzilla</t>
+        </is>
+      </c>
+      <c r="E556" t="inlineStr">
+        <is>
+          <t>3:31</t>
+        </is>
+      </c>
+      <c r="F556" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B557" t="n">
+        <v>3</v>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>Jay-Z &amp; Kanye West</t>
+        </is>
+      </c>
+      <c r="D557" t="inlineStr">
+        <is>
+          <t>Ni**as in Paris</t>
+        </is>
+      </c>
+      <c r="E557" t="inlineStr">
+        <is>
+          <t>3:39</t>
+        </is>
+      </c>
+      <c r="F557" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B558" t="n">
+        <v>4</v>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>Eminem</t>
+        </is>
+      </c>
+      <c r="D558" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="E558" t="inlineStr">
+        <is>
+          <t>4:11</t>
+        </is>
+      </c>
+      <c r="F558" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B559" t="n">
+        <v>5</v>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>Wiz Khalifa</t>
+        </is>
+      </c>
+      <c r="D559" t="inlineStr">
+        <is>
+          <t>Black and Yellow</t>
+        </is>
+      </c>
+      <c r="E559" t="inlineStr">
+        <is>
+          <t>3:37</t>
+        </is>
+      </c>
+      <c r="F559" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B560" t="n">
+        <v>6</v>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>Kanye West</t>
+        </is>
+      </c>
+      <c r="D560" t="inlineStr">
+        <is>
+          <t>Stronger</t>
+        </is>
+      </c>
+      <c r="E560" t="inlineStr">
+        <is>
+          <t>5:12</t>
+        </is>
+      </c>
+      <c r="F560" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B561" t="n">
+        <v>7</v>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>50 Cent feat. Eminem &amp; Tony Yayo</t>
+        </is>
+      </c>
+      <c r="D561" t="inlineStr">
+        <is>
+          <t>Patiently Waiting</t>
+        </is>
+      </c>
+      <c r="E561" t="inlineStr">
+        <is>
+          <t>4:48</t>
+        </is>
+      </c>
+      <c r="F561" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B562" t="n">
+        <v>8</v>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>M.O.P.</t>
+        </is>
+      </c>
+      <c r="D562" t="inlineStr">
+        <is>
+          <t>Ante Up</t>
+        </is>
+      </c>
+      <c r="E562" t="inlineStr">
+        <is>
+          <t>3:56</t>
+        </is>
+      </c>
+      <c r="F562" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B563" t="n">
+        <v>9</v>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>Lil Wayne feat. Cory Gunz</t>
+        </is>
+      </c>
+      <c r="D563" t="inlineStr">
+        <is>
+          <t>6 Foot 7 Foot</t>
+        </is>
+      </c>
+      <c r="E563" t="inlineStr">
+        <is>
+          <t>4:09</t>
+        </is>
+      </c>
+      <c r="F563" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B564" t="n">
+        <v>10</v>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>Bad Meets Evil</t>
+        </is>
+      </c>
+      <c r="D564" t="inlineStr">
+        <is>
+          <t>Fast Lane</t>
+        </is>
+      </c>
+      <c r="E564" t="inlineStr">
+        <is>
+          <t>4:10</t>
+        </is>
+      </c>
+      <c r="F564" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B565" t="n">
+        <v>11</v>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>Macklemore &amp; Ryan Lewis feat. Ray Dalton</t>
+        </is>
+      </c>
+      <c r="D565" t="inlineStr">
+        <is>
+          <t>Can't Hold Us</t>
+        </is>
+      </c>
+      <c r="E565" t="inlineStr">
+        <is>
+          <t>4:18</t>
+        </is>
+      </c>
+      <c r="F565" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B566" t="n">
+        <v>12</v>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>Eminem feat. Rihanna</t>
+        </is>
+      </c>
+      <c r="D566" t="inlineStr">
+        <is>
+          <t>The Monster</t>
+        </is>
+      </c>
+      <c r="E566" t="inlineStr">
+        <is>
+          <t>4:10</t>
+        </is>
+      </c>
+      <c r="F566" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B567" t="n">
+        <v>13</v>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>Flo Rida feat. T-Pain</t>
+        </is>
+      </c>
+      <c r="D567" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E567" t="inlineStr">
+        <is>
+          <t>3:50</t>
+        </is>
+      </c>
+      <c r="F567" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B568" t="n">
+        <v>14</v>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>J-Kwon</t>
+        </is>
+      </c>
+      <c r="D568" t="inlineStr">
+        <is>
+          <t>Tipsy</t>
+        </is>
+      </c>
+      <c r="E568" t="inlineStr">
+        <is>
+          <t>4:04</t>
+        </is>
+      </c>
+      <c r="F568" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B569" t="n">
+        <v>15</v>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>D12</t>
+        </is>
+      </c>
+      <c r="D569" t="inlineStr">
+        <is>
+          <t>Purple Pills</t>
+        </is>
+      </c>
+      <c r="E569" t="inlineStr">
+        <is>
+          <t>5:00</t>
+        </is>
+      </c>
+      <c r="F569" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B570" t="n">
+        <v>16</v>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>The Game feat. 50 Cent</t>
+        </is>
+      </c>
+      <c r="D570" t="inlineStr">
+        <is>
+          <t>Hate It or Love It</t>
+        </is>
+      </c>
+      <c r="E570" t="inlineStr">
+        <is>
+          <t>3:26</t>
+        </is>
+      </c>
+      <c r="F570" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B571" t="n">
+        <v>17</v>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>Nelly feat. P. Diddy &amp; Murphy Lee</t>
+        </is>
+      </c>
+      <c r="D571" t="inlineStr">
+        <is>
+          <t>Shake Ya Tailfeather</t>
+        </is>
+      </c>
+      <c r="E571" t="inlineStr">
+        <is>
+          <t>4:53</t>
+        </is>
+      </c>
+      <c r="F571" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B572" t="n">
+        <v>18</v>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>Eminem</t>
+        </is>
+      </c>
+      <c r="D572" t="inlineStr">
+        <is>
+          <t>Just Lose It</t>
+        </is>
+      </c>
+      <c r="E572" t="inlineStr">
+        <is>
+          <t>4:08</t>
+        </is>
+      </c>
+      <c r="F572" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B573" t="n">
+        <v>19</v>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>Ludacris</t>
+        </is>
+      </c>
+      <c r="D573" t="inlineStr">
+        <is>
+          <t>Get Back</t>
+        </is>
+      </c>
+      <c r="E573" t="inlineStr">
+        <is>
+          <t>4:30</t>
+        </is>
+      </c>
+      <c r="F573" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B574" t="n">
+        <v>20</v>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>Clipse</t>
+        </is>
+      </c>
+      <c r="D574" t="inlineStr">
+        <is>
+          <t>Grindin'</t>
+        </is>
+      </c>
+      <c r="E574" t="inlineStr">
+        <is>
+          <t>4:30</t>
+        </is>
+      </c>
+      <c r="F574" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B575" t="n">
+        <v>21</v>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>P. Diddy feat. Black Rob &amp; Mark Curry</t>
+        </is>
+      </c>
+      <c r="D575" t="inlineStr">
+        <is>
+          <t>Bad Boy for Life</t>
+        </is>
+      </c>
+      <c r="E575" t="inlineStr">
+        <is>
+          <t>3:42</t>
+        </is>
+      </c>
+      <c r="F575" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B576" t="n">
+        <v>22</v>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>Eminem feat. Dr. Dre</t>
+        </is>
+      </c>
+      <c r="D576" t="inlineStr">
+        <is>
+          <t>Guilty Conscience</t>
+        </is>
+      </c>
+      <c r="E576" t="inlineStr">
+        <is>
+          <t>3:19</t>
+        </is>
+      </c>
+      <c r="F576" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B577" t="n">
+        <v>23</v>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>Cam'ron feat. Juelz Santana</t>
+        </is>
+      </c>
+      <c r="D577" t="inlineStr">
+        <is>
+          <t>Oh Boy</t>
+        </is>
+      </c>
+      <c r="E577" t="inlineStr">
+        <is>
+          <t>3:34</t>
+        </is>
+      </c>
+      <c r="F577" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B578" t="n">
+        <v>24</v>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>50 Cent feat. Justin Timberlake &amp; Timbaland</t>
+        </is>
+      </c>
+      <c r="D578" t="inlineStr">
+        <is>
+          <t>Ayo Technology</t>
+        </is>
+      </c>
+      <c r="E578" t="inlineStr">
+        <is>
+          <t>4:07</t>
+        </is>
+      </c>
+      <c r="F578" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B579" t="n">
+        <v>25</v>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>Akon feat. Eminem</t>
+        </is>
+      </c>
+      <c r="D579" t="inlineStr">
+        <is>
+          <t>Smack That</t>
+        </is>
+      </c>
+      <c r="E579" t="inlineStr">
+        <is>
+          <t>3:33</t>
+        </is>
+      </c>
+      <c r="F579" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B580" t="n">
+        <v>26</v>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>Jim Jones</t>
+        </is>
+      </c>
+      <c r="D580" t="inlineStr">
+        <is>
+          <t>We Fly High</t>
+        </is>
+      </c>
+      <c r="E580" t="inlineStr">
+        <is>
+          <t>4:01</t>
+        </is>
+      </c>
+      <c r="F580" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B581" t="n">
+        <v>27</v>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>G-Unit</t>
+        </is>
+      </c>
+      <c r="D581" t="inlineStr">
+        <is>
+          <t>Stunt 101</t>
+        </is>
+      </c>
+      <c r="E581" t="inlineStr">
+        <is>
+          <t>4:04</t>
+        </is>
+      </c>
+      <c r="F581" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B582" t="n">
+        <v>28</v>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>Sir Mix-a-Lot</t>
+        </is>
+      </c>
+      <c r="D582" t="inlineStr">
+        <is>
+          <t>Baby Got Back</t>
+        </is>
+      </c>
+      <c r="E582" t="inlineStr">
+        <is>
+          <t>4:22</t>
+        </is>
+      </c>
+      <c r="F582" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B583" t="n">
+        <v>29</v>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>Vanilla Ice</t>
+        </is>
+      </c>
+      <c r="D583" t="inlineStr">
+        <is>
+          <t>Ice Ice Baby</t>
+        </is>
+      </c>
+      <c r="E583" t="inlineStr">
+        <is>
+          <t>4:31</t>
+        </is>
+      </c>
+      <c r="F583" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B584" t="n">
+        <v>30</v>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>MC Hammer</t>
+        </is>
+      </c>
+      <c r="D584" t="inlineStr">
+        <is>
+          <t>U Can't Touch This</t>
+        </is>
+      </c>
+      <c r="E584" t="inlineStr">
+        <is>
+          <t>4:17</t>
+        </is>
+      </c>
+      <c r="F584" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B585" t="n">
+        <v>31</v>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>Kris Kross</t>
+        </is>
+      </c>
+      <c r="D585" t="inlineStr">
+        <is>
+          <t>Jump</t>
+        </is>
+      </c>
+      <c r="E585" t="inlineStr">
+        <is>
+          <t>3:16</t>
+        </is>
+      </c>
+      <c r="F585" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B586" t="n">
+        <v>32</v>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>Naughty by Nature</t>
+        </is>
+      </c>
+      <c r="D586" t="inlineStr">
+        <is>
+          <t>Hip Hop Hooray</t>
+        </is>
+      </c>
+      <c r="E586" t="inlineStr">
+        <is>
+          <t>4:26</t>
+        </is>
+      </c>
+      <c r="F586" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B587" t="n">
+        <v>33</v>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>Run-DMC</t>
+        </is>
+      </c>
+      <c r="D587" t="inlineStr">
+        <is>
+          <t>It's Tricky</t>
+        </is>
+      </c>
+      <c r="E587" t="inlineStr">
+        <is>
+          <t>3:03</t>
+        </is>
+      </c>
+      <c r="F587" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B588" t="n">
+        <v>34</v>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>Beastie Boys</t>
+        </is>
+      </c>
+      <c r="D588" t="inlineStr">
+        <is>
+          <t>Brass Monkey</t>
+        </is>
+      </c>
+      <c r="E588" t="inlineStr">
+        <is>
+          <t>2:37</t>
+        </is>
+      </c>
+      <c r="F588" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B589" t="n">
+        <v>35</v>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>Rob Base &amp; DJ E-Z Rock</t>
+        </is>
+      </c>
+      <c r="D589" t="inlineStr">
+        <is>
+          <t>It Takes Two</t>
+        </is>
+      </c>
+      <c r="E589" t="inlineStr">
+        <is>
+          <t>4:57</t>
+        </is>
+      </c>
+      <c r="F589" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B590" t="n">
+        <v>36</v>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>Luniz feat. Michael Marshall</t>
+        </is>
+      </c>
+      <c r="D590" t="inlineStr">
+        <is>
+          <t>I Got 5 on It</t>
+        </is>
+      </c>
+      <c r="E590" t="inlineStr">
+        <is>
+          <t>4:14</t>
+        </is>
+      </c>
+      <c r="F590" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B591" t="n">
+        <v>37</v>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>Eminem feat. Dido</t>
+        </is>
+      </c>
+      <c r="D591" t="inlineStr">
+        <is>
+          <t>Stan</t>
+        </is>
+      </c>
+      <c r="E591" t="inlineStr">
+        <is>
+          <t>6:44</t>
+        </is>
+      </c>
+      <c r="F591" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B592" t="n">
+        <v>38</v>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>Xzibit</t>
+        </is>
+      </c>
+      <c r="D592" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E592" t="inlineStr">
+        <is>
+          <t>3:47</t>
+        </is>
+      </c>
+      <c r="F592" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B593" t="n">
+        <v>39</v>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>Fat Joe &amp; Remy Ma feat. French Montana &amp; Infared</t>
+        </is>
+      </c>
+      <c r="D593" t="inlineStr">
+        <is>
+          <t>All the Way Up</t>
+        </is>
+      </c>
+      <c r="E593" t="inlineStr">
+        <is>
+          <t>3:36</t>
+        </is>
+      </c>
+      <c r="F593" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B594" t="n">
+        <v>40</v>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>Rick Ross feat. Styles P</t>
+        </is>
+      </c>
+      <c r="D594" t="inlineStr">
+        <is>
+          <t>B.M.F. (Blowin' Money Fast)</t>
+        </is>
+      </c>
+      <c r="E594" t="inlineStr">
+        <is>
+          <t>4:15</t>
+        </is>
+      </c>
+      <c r="F594" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B595" t="n">
+        <v>41</v>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>Eminem</t>
+        </is>
+      </c>
+      <c r="D595" t="inlineStr">
+        <is>
+          <t>Like Toy Soldiers</t>
+        </is>
+      </c>
+      <c r="E595" t="inlineStr">
+        <is>
+          <t>4:56</t>
+        </is>
+      </c>
+      <c r="F595" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B596" t="n">
+        <v>42</v>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>Asher Roth</t>
+        </is>
+      </c>
+      <c r="D596" t="inlineStr">
+        <is>
+          <t>I Love College</t>
+        </is>
+      </c>
+      <c r="E596" t="inlineStr">
+        <is>
+          <t>4:01</t>
+        </is>
+      </c>
+      <c r="F596" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B597" t="n">
+        <v>43</v>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>Soulja Boy</t>
+        </is>
+      </c>
+      <c r="D597" t="inlineStr">
+        <is>
+          <t>Crank That (Soulja Boy)</t>
+        </is>
+      </c>
+      <c r="E597" t="inlineStr">
+        <is>
+          <t>3:42</t>
+        </is>
+      </c>
+      <c r="F597" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B598" t="n">
+        <v>44</v>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>Macklemore &amp; Ryan Lewis feat. Wanz</t>
+        </is>
+      </c>
+      <c r="D598" t="inlineStr">
+        <is>
+          <t>Thrift Shop</t>
+        </is>
+      </c>
+      <c r="E598" t="inlineStr">
+        <is>
+          <t>3:55</t>
+        </is>
+      </c>
+      <c r="F598" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B599" t="n">
+        <v>45</v>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>Jay-Z feat. Eminem</t>
+        </is>
+      </c>
+      <c r="D599" t="inlineStr">
+        <is>
+          <t>Renegade</t>
+        </is>
+      </c>
+      <c r="E599" t="inlineStr">
+        <is>
+          <t>5:38</t>
+        </is>
+      </c>
+      <c r="F599" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B600" t="n">
+        <v>46</v>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>Travis Scott</t>
+        </is>
+      </c>
+      <c r="D600" t="inlineStr">
+        <is>
+          <t>SICKO MODE</t>
+        </is>
+      </c>
+      <c r="E600" t="inlineStr">
+        <is>
+          <t>5:12</t>
+        </is>
+      </c>
+      <c r="F600" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B601" t="n">
+        <v>47</v>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>Post Malone feat. Quavo</t>
+        </is>
+      </c>
+      <c r="D601" t="inlineStr">
+        <is>
+          <t>Congratulations</t>
+        </is>
+      </c>
+      <c r="E601" t="inlineStr">
+        <is>
+          <t>3:40</t>
+        </is>
+      </c>
+      <c r="F601" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B602" t="n">
+        <v>48</v>
+      </c>
+      <c r="C602" t="inlineStr">
+        <is>
+          <t>Drake feat. Lil Wayne</t>
+        </is>
+      </c>
+      <c r="D602" t="inlineStr">
+        <is>
+          <t>The Motto</t>
+        </is>
+      </c>
+      <c r="E602" t="inlineStr">
+        <is>
+          <t>3:01</t>
+        </is>
+      </c>
+      <c r="F602" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B603" t="n">
+        <v>49</v>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>Kanye West feat. Rihanna &amp; Kid Cudi</t>
+        </is>
+      </c>
+      <c r="D603" t="inlineStr">
+        <is>
+          <t>All of the Lights</t>
+        </is>
+      </c>
+      <c r="E603" t="inlineStr">
+        <is>
+          <t>4:59</t>
+        </is>
+      </c>
+      <c r="F603" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B604" t="n">
+        <v>50</v>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>Big Sean feat. E-40</t>
+        </is>
+      </c>
+      <c r="D604" t="inlineStr">
+        <is>
+          <t>I Don't Fuck with You</t>
+        </is>
+      </c>
+      <c r="E604" t="inlineStr">
+        <is>
+          <t>4:44</t>
+        </is>
+      </c>
+      <c r="F604" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B605" t="n">
+        <v>51</v>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>Kanye West</t>
+        </is>
+      </c>
+      <c r="D605" t="inlineStr">
+        <is>
+          <t>Heartless</t>
+        </is>
+      </c>
+      <c r="E605" t="inlineStr">
+        <is>
+          <t>3:31</t>
+        </is>
+      </c>
+      <c r="F605" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B606" t="n">
+        <v>52</v>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>Eminem feat. Lil Wayne</t>
+        </is>
+      </c>
+      <c r="D606" t="inlineStr">
+        <is>
+          <t>No Love</t>
+        </is>
+      </c>
+      <c r="E606" t="inlineStr">
+        <is>
+          <t>5:00</t>
+        </is>
+      </c>
+      <c r="F606" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B607" t="n">
+        <v>53</v>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>Kid Cudi</t>
+        </is>
+      </c>
+      <c r="D607" t="inlineStr">
+        <is>
+          <t>Day 'N' Nite</t>
+        </is>
+      </c>
+      <c r="E607" t="inlineStr">
+        <is>
+          <t>3:42</t>
+        </is>
+      </c>
+      <c r="F607" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B608" t="n">
+        <v>54</v>
+      </c>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>Drake</t>
+        </is>
+      </c>
+      <c r="D608" t="inlineStr">
+        <is>
+          <t>Started From the Bottom</t>
+        </is>
+      </c>
+      <c r="E608" t="inlineStr">
+        <is>
+          <t>2:53</t>
+        </is>
+      </c>
+      <c r="F608" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B609" t="n">
+        <v>55</v>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>DJ Khaled feat. Drake, Rick Ross &amp; Lil Wayne</t>
+        </is>
+      </c>
+      <c r="D609" t="inlineStr">
+        <is>
+          <t>I'm On One</t>
+        </is>
+      </c>
+      <c r="E609" t="inlineStr">
+        <is>
+          <t>4:56</t>
+        </is>
+      </c>
+      <c r="F609" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B610" t="n">
+        <v>56</v>
+      </c>
+      <c r="C610" t="inlineStr">
+        <is>
+          <t>B.o.B feat. Hayley Williams &amp; Eminem</t>
+        </is>
+      </c>
+      <c r="D610" t="inlineStr">
+        <is>
+          <t>Airplanes, Pt. II</t>
+        </is>
+      </c>
+      <c r="E610" t="inlineStr">
+        <is>
+          <t>4:20</t>
+        </is>
+      </c>
+      <c r="F610" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B611" t="n">
+        <v>57</v>
+      </c>
+      <c r="C611" t="inlineStr">
+        <is>
+          <t>Jay-Z feat. Rihanna &amp; Kanye West</t>
+        </is>
+      </c>
+      <c r="D611" t="inlineStr">
+        <is>
+          <t>Run This Town</t>
+        </is>
+      </c>
+      <c r="E611" t="inlineStr">
+        <is>
+          <t>4:27</t>
+        </is>
+      </c>
+      <c r="F611" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B612" t="n">
+        <v>58</v>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>Nelly</t>
+        </is>
+      </c>
+      <c r="D612" t="inlineStr">
+        <is>
+          <t>E.I.</t>
+        </is>
+      </c>
+      <c r="E612" t="inlineStr">
+        <is>
+          <t>4:47</t>
+        </is>
+      </c>
+      <c r="F612" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B613" t="n">
+        <v>59</v>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>Juvenile feat. Soulja Slim</t>
+        </is>
+      </c>
+      <c r="D613" t="inlineStr">
+        <is>
+          <t>Slow Motion</t>
+        </is>
+      </c>
+      <c r="E613" t="inlineStr">
+        <is>
+          <t>4:10</t>
+        </is>
+      </c>
+      <c r="F613" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B614" t="n">
+        <v>60</v>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>Outkast</t>
+        </is>
+      </c>
+      <c r="D614" t="inlineStr">
+        <is>
+          <t>Roses</t>
+        </is>
+      </c>
+      <c r="E614" t="inlineStr">
+        <is>
+          <t>6:09</t>
+        </is>
+      </c>
+      <c r="F614" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B615" t="n">
+        <v>61</v>
+      </c>
+      <c r="C615" t="inlineStr">
+        <is>
+          <t>Linkin Park &amp; Jay-Z</t>
+        </is>
+      </c>
+      <c r="D615" t="inlineStr">
+        <is>
+          <t>Numb / Encore</t>
+        </is>
+      </c>
+      <c r="E615" t="inlineStr">
+        <is>
+          <t>3:25</t>
+        </is>
+      </c>
+      <c r="F615" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B616" t="n">
+        <v>62</v>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>Papa Roach</t>
+        </is>
+      </c>
+      <c r="D616" t="inlineStr">
+        <is>
+          <t>Last Resort</t>
+        </is>
+      </c>
+      <c r="E616" t="inlineStr">
+        <is>
+          <t>3:20</t>
+        </is>
+      </c>
+      <c r="F616" t="inlineStr">
+        <is>
+          <t>Rock</t>
+        </is>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B617" t="n">
+        <v>63</v>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>Too $hort</t>
+        </is>
+      </c>
+      <c r="D617" t="inlineStr">
+        <is>
+          <t>Blow the Whistle</t>
+        </is>
+      </c>
+      <c r="E617" t="inlineStr">
+        <is>
+          <t>2:46</t>
+        </is>
+      </c>
+      <c r="F617" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B618" t="n">
+        <v>64</v>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>Bad Meets Evil feat. Bruno Mars</t>
+        </is>
+      </c>
+      <c r="D618" t="inlineStr">
+        <is>
+          <t>Lighters</t>
+        </is>
+      </c>
+      <c r="E618" t="inlineStr">
+        <is>
+          <t>5:04</t>
+        </is>
+      </c>
+      <c r="F618" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B619" t="n">
+        <v>65</v>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>Drake feat. Kanye West, Lil Wayne &amp; Eminem</t>
+        </is>
+      </c>
+      <c r="D619" t="inlineStr">
+        <is>
+          <t>Forever</t>
+        </is>
+      </c>
+      <c r="E619" t="inlineStr">
+        <is>
+          <t>5:57</t>
+        </is>
+      </c>
+      <c r="F619" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B620" t="n">
+        <v>66</v>
+      </c>
+      <c r="C620" t="inlineStr">
+        <is>
+          <t>Eminem feat. Rihanna</t>
+        </is>
+      </c>
+      <c r="D620" t="inlineStr">
+        <is>
+          <t>Love the Way You Lie</t>
+        </is>
+      </c>
+      <c r="E620" t="inlineStr">
+        <is>
+          <t>4:23</t>
+        </is>
+      </c>
+      <c r="F620" t="inlineStr">
+        <is>
+          <t>Rap</t>
+        </is>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="inlineStr">
+        <is>
+          <t>The Ride Up</t>
+        </is>
+      </c>
+      <c r="B621" t="n">
+        <v>67</v>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>Eminem</t>
+        </is>
+      </c>
+      <c r="D621" t="inlineStr">
+        <is>
+          <t>Not Afraid</t>
+        </is>
+      </c>
+      <c r="E621" t="inlineStr">
+        <is>
+          <t>4:08</t>
+        </is>
+      </c>
+      <c r="F621" t="inlineStr">
+        <is>
+          <t>Rap</t>
         </is>
       </c>
     </row>

</xml_diff>